<commit_message>
Fix Excel chart overlap and extend screener filters
</commit_message>
<xml_diff>
--- a/exports/preview_screen.xlsx
+++ b/exports/preview_screen.xlsx
@@ -768,10 +768,10 @@
         <v>213500</v>
       </c>
       <c r="E9" s="11" t="n">
-        <v>-0.47</v>
+        <v>-0.4662004662004662</v>
       </c>
       <c r="F9" s="10" t="n">
-        <v>12481804.8</v>
+        <v>12481805</v>
       </c>
       <c r="G9" s="12" t="n">
         <v>9.58</v>
@@ -827,10 +827,10 @@
         <v>1263000</v>
       </c>
       <c r="E10" s="19" t="n">
-        <v>3.27</v>
+        <v>3.270645952575634</v>
       </c>
       <c r="F10" s="18" t="n">
-        <v>9226118.6</v>
+        <v>9226119</v>
       </c>
       <c r="G10" s="20" t="n">
         <v>5.63</v>
@@ -1208,10 +1208,10 @@
         <v>153000</v>
       </c>
       <c r="E17" s="11" t="n">
-        <v>-3.29</v>
+        <v>-3.286978508217446</v>
       </c>
       <c r="F17" s="10" t="n">
-        <v>542672.2</v>
+        <v>542672</v>
       </c>
       <c r="G17" s="12" t="n">
         <v>9.140000000000001</v>
@@ -1487,10 +1487,10 @@
         <v>88000</v>
       </c>
       <c r="E22" s="23" t="n">
-        <v>-2.55</v>
+        <v>-2.547065337763012</v>
       </c>
       <c r="F22" s="18" t="n">
-        <v>413116.2</v>
+        <v>413116</v>
       </c>
       <c r="G22" s="20" t="n">
         <v>7.88</v>

</xml_diff>